<commit_message>
Fix bulk registration names and identity search
</commit_message>
<xml_diff>
--- a/public/templates/pcc-bulk-registration-template.xlsx
+++ b/public/templates/pcc-bulk-registration-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R21affd50927f4557"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R15b73fb968474c76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -167,7 +167,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top"/>
@@ -287,6 +287,27 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -514,53 +535,54 @@
   <x:cols>
     <x:col min="1" max="1" width="6" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="2" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="8" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="3.25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="2.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="6.130000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="20" customHeight="1">
       <x:c r="A1" s="15" t="str">
         <x:v>PCC Registration Platform bulk entry sheet</x:v>
       </x:c>
-      <x:c r="B1" s="15"/>
-      <x:c r="C1" s="15"/>
-      <x:c r="D1" s="15"/>
+      <x:c r="B1" s="15" t="str"/>
+      <x:c r="C1" s="15" t="str"/>
+      <x:c r="D1" s="15" t="str"/>
       <x:c r="E1" s="17" t="str">
         <x:v>polokwanechessclub.co.za</x:v>
       </x:c>
-      <x:c r="F1" s="17"/>
-      <x:c r="G1" s="17"/>
-      <x:c r="H1" s="17"/>
+      <x:c r="F1" s="17" t="str"/>
+      <x:c r="G1" s="17" t="str"/>
+      <x:c r="H1" s="17" t="str"/>
     </x:row>
     <x:row r="2" ht="20" customHeight="1">
       <x:c r="A2" s="18" t="str">
         <x:v>Tournament Name &amp; Date:</x:v>
       </x:c>
-      <x:c r="B2" s="19"/>
-      <x:c r="C2" s="19"/>
+      <x:c r="B2" s="19" t="str"/>
+      <x:c r="C2" s="19" t="str"/>
       <x:c r="D2" s="20" t="str">
         <x:v>Enter tournament name and date here</x:v>
       </x:c>
-      <x:c r="E2" s="20"/>
-      <x:c r="F2" s="20"/>
-      <x:c r="G2" s="20"/>
-      <x:c r="H2" s="20"/>
+      <x:c r="E2" s="20" t="str"/>
+      <x:c r="F2" s="20" t="str"/>
+      <x:c r="G2" s="20" t="str"/>
+      <x:c r="H2" s="20" t="str"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="22" t="str">
-        <x:v>Complete one player per row. Required: Name and Date of birth. Optional: FED, Rating, Club/City and Gender.</x:v>
-      </x:c>
-      <x:c r="B3" s="22"/>
-      <x:c r="C3" s="22"/>
-      <x:c r="D3" s="22"/>
-      <x:c r="E3" s="22"/>
-      <x:c r="F3" s="22"/>
-      <x:c r="G3" s="22"/>
-      <x:c r="H3" s="22"/>
+        <x:v>Use separate First names and Surname columns. Do not enter surname-first names or commas.</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str"/>
+      <x:c r="C3" s="22" t="str"/>
+      <x:c r="D3" s="22" t="str"/>
+      <x:c r="E3" s="22" t="str"/>
+      <x:c r="F3" s="22" t="str"/>
+      <x:c r="G3" s="22" t="str"/>
+      <x:c r="H3" s="22" t="str"/>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
       <x:c r="A4" s="18" t="str">
@@ -579,22 +601,25 @@
         <x:v>No.</x:v>
       </x:c>
       <x:c r="B5" s="36"/>
-      <x:c r="C5" s="36" t="str">
-        <x:v>Name</x:v>
-      </x:c>
-      <x:c r="D5" s="37" t="str">
+      <x:c r="C5" s="50" t="str">
+        <x:v>First names</x:v>
+      </x:c>
+      <x:c r="D5" s="51" t="str">
+        <x:v>Surname</x:v>
+      </x:c>
+      <x:c r="E5" s="50" t="str">
         <x:v>Date of birth</x:v>
       </x:c>
-      <x:c r="E5" s="36" t="str">
+      <x:c r="F5" s="52" t="str">
         <x:v>FED</x:v>
       </x:c>
-      <x:c r="F5" s="38" t="str">
+      <x:c r="G5" s="50" t="str">
         <x:v>Rtg</x:v>
       </x:c>
-      <x:c r="G5" s="36" t="str">
+      <x:c r="H5" s="50" t="str">
         <x:v>Club/City</x:v>
       </x:c>
-      <x:c r="H5" s="36" t="str">
+      <x:c r="I5" s="56" t="str">
         <x:v>Gender</x:v>
       </x:c>
     </x:row>
@@ -603,42 +628,65 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B6" s="45"/>
-      <x:c r="C6" s="45"/>
-      <x:c r="D6" s="48"/>
-      <x:c r="E6" s="45" t="str">
-        <x:v>RSA</x:v>
-      </x:c>
-      <x:c r="F6" s="49"/>
-      <x:c r="G6" s="45"/>
-      <x:c r="H6" s="45"/>
+      <x:c r="C6" s="53" t="str">
+        <x:v>Thabo James</x:v>
+      </x:c>
+      <x:c r="D6" s="54" t="str">
+        <x:v>Van der Merwe</x:v>
+      </x:c>
+      <x:c r="E6" s="53" t="str">
+        <x:v>2012-04-05</x:v>
+      </x:c>
+      <x:c r="F6" s="55" t="str">
+        <x:v>RSA</x:v>
+      </x:c>
+      <x:c r="G6" s="53" t="str"/>
+      <x:c r="H6" s="53" t="str">
+        <x:v>Example school</x:v>
+      </x:c>
+      <x:c r="I6" s="56" t="str">
+        <x:v>Male</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="45" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="45"/>
-      <x:c r="C7" s="45"/>
-      <x:c r="D7" s="48"/>
-      <x:c r="E7" s="45" t="str">
-        <x:v>RSA</x:v>
-      </x:c>
-      <x:c r="F7" s="49"/>
-      <x:c r="G7" s="45"/>
-      <x:c r="H7" s="45"/>
+      <x:c r="C7" s="53" t="str">
+        <x:v>Basetsana</x:v>
+      </x:c>
+      <x:c r="D7" s="54" t="str">
+        <x:v>Sedibe</x:v>
+      </x:c>
+      <x:c r="E7" s="53" t="str">
+        <x:v>2013-01-03</x:v>
+      </x:c>
+      <x:c r="F7" s="55" t="str">
+        <x:v>RSA</x:v>
+      </x:c>
+      <x:c r="G7" s="53" t="str"/>
+      <x:c r="H7" s="53" t="str">
+        <x:v>Example school</x:v>
+      </x:c>
+      <x:c r="I7" s="56" t="str">
+        <x:v>Female</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="45" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="45"/>
-      <x:c r="C8" s="45"/>
-      <x:c r="D8" s="48"/>
-      <x:c r="E8" s="45" t="str">
-        <x:v>RSA</x:v>
-      </x:c>
-      <x:c r="F8" s="49"/>
-      <x:c r="G8" s="45"/>
-      <x:c r="H8" s="45"/>
+      <x:c r="C8" s="53" t="str"/>
+      <x:c r="D8" s="54" t="str"/>
+      <x:c r="E8" s="53" t="str"/>
+      <x:c r="F8" s="55" t="str">
+        <x:v>RSA</x:v>
+      </x:c>
+      <x:c r="G8" s="53" t="str"/>
+      <x:c r="H8" s="53" t="str"/>
+      <x:c r="I8" s="56" t="str"/>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="45" t="n">
@@ -1247,11 +1295,11 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="R31e786796af742fc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1" r:id="Rbbc05c1bf0764419"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E1" r:id="Rc479c96b2bdb4fb4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1" r:id="R3fdc1f81776d4972"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G1" r:id="Rd279fa5a16ba4db9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="R022c3829baaf4815"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1" r:id="R8e97fab33f384194"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E1" r:id="R95079d2c8c9546b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1" r:id="Re152f8895bb44ec6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G1" r:id="Ra12c8a5cb89342d2"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>